<commit_message>
items import | ccolor size code
</commit_message>
<xml_diff>
--- a/public/formats/item_color_size.xlsx
+++ b/public/formats/item_color_size.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\sdrimsac-tenant\public\formats\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\laragon\www\sdrimsac-tenant\public\formats\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Código Interno (Producto)</t>
   </si>
@@ -48,6 +48,15 @@
   </si>
   <si>
     <t>Precio</t>
+  </si>
+  <si>
+    <t>Codigo talla color</t>
+  </si>
+  <si>
+    <t>100030-1</t>
+  </si>
+  <si>
+    <t>100030-2</t>
   </si>
 </sst>
 </file>
@@ -365,62 +374,73 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.28515625" customWidth="1"/>
+    <col min="3" max="3" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>100030</v>
       </c>
       <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>34</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>10</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>100030</v>
       </c>
       <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>5</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>3</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>3</v>
       </c>
     </row>

</xml_diff>